<commit_message>
Unify cross-page search and refresh criticism data and figures
</commit_message>
<xml_diff>
--- a/criticism.xlsx
+++ b/criticism.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10315"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/qiyuchen/Documents/挑战杯/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADEE21BB-AA00-0A4A-9CD9-C5747F91DFFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="9952" windowHeight="9555" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="23480" windowHeight="15400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="eval_edges" sheetId="1" r:id="rId1"/>
@@ -30,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="204">
   <si>
     <t>edge_id</t>
   </si>
@@ -356,9 +362,6 @@
     <t>遁其天然，牵于俗情，如被刑然。</t>
   </si>
   <si>
-    <t>EDGE0025</t>
-  </si>
-  <si>
     <t>E12</t>
   </si>
   <si>
@@ -639,23 +642,23 @@
   </si>
   <si>
     <t>eval_edges=24, ref_notes=31, pending=0</t>
+  </si>
+  <si>
+    <t>REF0030</t>
+  </si>
+  <si>
+    <t>EDGE0016</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="23">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="宋体"/>
+      <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -670,160 +673,29 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
-      <charset val="134"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="等线"/>
+      <family val="4"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -836,194 +708,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -1031,253 +717,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1291,62 +735,21 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="49">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1631,14 +1034,14 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:XFD26"/>
-  <sheetFormatPr defaultColWidth="8.83185840707965" defaultRowHeight="13.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -1683,7 +1086,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" ht="27" spans="1:10">
+    <row r="2" spans="1:10" ht="32">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -1715,8 +1118,8 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:10" customFormat="1" ht="16">
+      <c r="A3" s="5" t="s">
         <v>18</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -1729,10 +1132,10 @@
         <v>143</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>22</v>
@@ -1747,7 +1150,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" customFormat="1" ht="16">
       <c r="A4" s="2" t="s">
         <v>25</v>
       </c>
@@ -1761,10 +1164,10 @@
         <v>143</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>22</v>
@@ -1773,45 +1176,45 @@
         <v>23</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="J4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:10" customFormat="1" ht="128">
+      <c r="A5" s="5" t="s">
         <v>28</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="C5" s="2">
         <v>1</v>
       </c>
       <c r="D5" s="2">
-        <v>143</v>
+        <v>193</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" ht="121.5" spans="1:10">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" customFormat="1" ht="144">
       <c r="A6" s="2" t="s">
         <v>32</v>
       </c>
@@ -1825,16 +1228,16 @@
         <v>193</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>31</v>
@@ -1843,8 +1246,8 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" ht="135" spans="1:10">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:10" customFormat="1" ht="32">
+      <c r="A7" s="5" t="s">
         <v>39</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -1857,10 +1260,10 @@
         <v>193</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>40</v>
@@ -1869,46 +1272,46 @@
         <v>41</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="J7" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="8" ht="27" spans="1:10">
+    <row r="8" spans="1:10" customFormat="1" ht="34">
       <c r="A8" s="2" t="s">
         <v>42</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="C8" s="2">
         <v>1</v>
       </c>
       <c r="D8" s="2">
-        <v>193</v>
+        <v>235</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>40</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J8" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="9" ht="31.5" spans="1:10">
-      <c r="A9" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" customFormat="1" ht="34">
+      <c r="A9" s="5" t="s">
         <v>45</v>
       </c>
       <c r="B9" s="2" t="s">
@@ -1921,10 +1324,10 @@
         <v>235</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>40</v>
@@ -1933,175 +1336,175 @@
         <v>49</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="J9" s="3" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="10" ht="31.5" spans="1:10">
+    <row r="10" spans="1:10" customFormat="1" ht="32">
       <c r="A10" s="2" t="s">
         <v>51</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="C10" s="2">
         <v>1</v>
       </c>
       <c r="D10" s="2">
-        <v>235</v>
+        <v>406</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="J10" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="11" ht="27" spans="1:10">
-      <c r="A11" s="2" t="s">
+      <c r="J10" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" customFormat="1" ht="32">
+      <c r="A11" s="5" t="s">
         <v>54</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C11" s="2">
         <v>1</v>
       </c>
       <c r="D11" s="2">
-        <v>406</v>
+        <v>510</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>56</v>
+        <v>20</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="J11" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="12" ht="27" spans="1:10">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" customFormat="1" ht="32">
       <c r="A12" s="2" t="s">
         <v>60</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C12" s="2">
         <v>1</v>
       </c>
       <c r="D12" s="2">
-        <v>510</v>
+        <v>515</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J12" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="13" ht="27" spans="1:10">
-      <c r="A13" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" customFormat="1" ht="32">
+      <c r="A13" s="5" t="s">
         <v>65</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C13" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13" s="2">
-        <v>515</v>
+        <v>149</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="J13" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="14" ht="27" spans="1:10">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" customFormat="1" ht="32">
       <c r="A14" s="2" t="s">
         <v>70</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C14" s="2">
         <v>2</v>
       </c>
       <c r="D14" s="2">
-        <v>149</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>36</v>
+        <v>185</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>76</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>16</v>
       </c>
       <c r="J14" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="15" ht="27" spans="1:10">
-      <c r="A15" s="2" t="s">
-        <v>70</v>
+        <v>79</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" customFormat="1" ht="32">
+      <c r="A15" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>75</v>
@@ -2113,10 +1516,10 @@
         <v>185</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>76</v>
+        <v>52</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>29</v>
@@ -2131,9 +1534,9 @@
         <v>79</v>
       </c>
     </row>
-    <row r="16" ht="27" spans="1:10">
+    <row r="16" spans="1:10" customFormat="1" ht="32">
       <c r="A16" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>75</v>
@@ -2144,11 +1547,11 @@
       <c r="D16" s="2">
         <v>185</v>
       </c>
-      <c r="E16" s="4" t="s">
-        <v>52</v>
+      <c r="E16" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>29</v>
@@ -2163,39 +1566,39 @@
         <v>79</v>
       </c>
     </row>
-    <row r="17" ht="27" spans="1:10 16384:16384">
-      <c r="A17" s="2" t="s">
-        <v>82</v>
+    <row r="17" spans="1:10 16384:16384" customFormat="1" ht="32">
+      <c r="A17" s="5" t="s">
+        <v>203</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="C17" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D17" s="2">
-        <v>185</v>
+        <v>9</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>16</v>
       </c>
       <c r="J17" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="18" ht="27" spans="1:10 16384:16384">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10 16384:16384" customFormat="1" ht="48">
       <c r="A18" s="2" t="s">
         <v>84</v>
       </c>
@@ -2209,10 +1612,10 @@
         <v>9</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>34</v>
+        <v>90</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>22</v>
@@ -2221,45 +1624,49 @@
         <v>87</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="J18" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="19" ht="40.5" spans="1:10 16384:16384">
-      <c r="A19" s="2" t="s">
+    <row r="19" spans="1:10 16384:16384" customFormat="1" ht="32">
+      <c r="A19" s="5" t="s">
         <v>89</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C19" s="2">
         <v>3</v>
       </c>
       <c r="D19" s="2">
-        <v>9</v>
+        <v>114</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>90</v>
+        <v>34</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="J19" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="20" ht="27" spans="1:10 16384:16384">
+        <v>96</v>
+      </c>
+      <c r="XFD19">
+        <f t="shared" ref="XFD19:XFD25" si="0">SUM(C19:XFC19)</f>
+        <v>117</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10 16384:16384" customFormat="1" ht="32">
       <c r="A20" s="2" t="s">
         <v>92</v>
       </c>
@@ -2273,10 +1680,10 @@
         <v>114</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>40</v>
@@ -2291,12 +1698,12 @@
         <v>96</v>
       </c>
       <c r="XFD20">
-        <f t="shared" ref="XFD20:XFD26" si="0">SUM(C20:XFC20)</f>
+        <f t="shared" si="0"/>
         <v>117</v>
       </c>
     </row>
-    <row r="21" ht="40.5" spans="1:10 16384:16384">
-      <c r="A21" s="2" t="s">
+    <row r="21" spans="1:10 16384:16384" customFormat="1" ht="32">
+      <c r="A21" s="5" t="s">
         <v>97</v>
       </c>
       <c r="B21" s="2" t="s">
@@ -2309,10 +1716,10 @@
         <v>114</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>29</v>
+        <v>100</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>40</v>
@@ -2331,7 +1738,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="22" ht="27" spans="1:10 16384:16384">
+    <row r="22" spans="1:10 16384:16384" customFormat="1" ht="32">
       <c r="A22" s="2" t="s">
         <v>99</v>
       </c>
@@ -2345,10 +1752,10 @@
         <v>114</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>100</v>
+        <v>26</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>40</v>
@@ -2367,8 +1774,8 @@
         <v>117</v>
       </c>
     </row>
-    <row r="23" ht="27" spans="1:10 16384:16384">
-      <c r="A23" s="2" t="s">
+    <row r="23" spans="1:10 16384:16384" customFormat="1" ht="32">
+      <c r="A23" s="5" t="s">
         <v>102</v>
       </c>
       <c r="B23" s="2" t="s">
@@ -2381,10 +1788,10 @@
         <v>114</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>26</v>
+        <v>90</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>40</v>
@@ -2403,7 +1810,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="24" ht="27" spans="1:10 16384:16384">
+    <row r="24" spans="1:10 16384:16384" customFormat="1" ht="32">
       <c r="A24" s="2" t="s">
         <v>104</v>
       </c>
@@ -2417,10 +1824,10 @@
         <v>114</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>90</v>
+        <v>43</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>40</v>
@@ -2439,94 +1846,58 @@
         <v>117</v>
       </c>
     </row>
-    <row r="25" ht="27" spans="1:10 16384:16384">
-      <c r="A25" s="2" t="s">
+    <row r="25" spans="1:10 16384:16384" customFormat="1" ht="64">
+      <c r="A25" s="5" t="s">
         <v>106</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>93</v>
+        <v>108</v>
       </c>
       <c r="C25" s="2">
         <v>3</v>
       </c>
       <c r="D25" s="2">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>16</v>
       </c>
       <c r="J25" t="s">
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="XFD25">
         <f t="shared" si="0"/>
-        <v>117</v>
-      </c>
-    </row>
-    <row r="26" ht="54" spans="1:10 16384:16384">
-      <c r="A26" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="C26" s="2">
-        <v>3</v>
-      </c>
-      <c r="D26" s="2">
-        <v>121</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="I26" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J26" t="s">
-        <v>112</v>
-      </c>
-      <c r="XFD26">
-        <f t="shared" si="0"/>
         <v>124</v>
       </c>
     </row>
+    <row r="26" spans="1:10 16384:16384" customFormat="1"/>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="I2:I1048576">
+    <dataValidation type="list" sqref="I2:I1048576" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:F30"/>
-  <sheetFormatPr defaultColWidth="8.83185840707965" defaultRowHeight="13.5" outlineLevelCol="5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:F31"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -2538,10 +1909,10 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>113</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>114</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2550,18 +1921,18 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="F1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:6" ht="16">
+      <c r="A2" s="2" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="2" t="s">
+      <c r="B2" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>118</v>
       </c>
       <c r="C2" s="2">
         <v>1</v>
@@ -2570,18 +1941,18 @@
         <v>143</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" customFormat="1" ht="16">
       <c r="A3" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C3" s="2">
         <v>1</v>
@@ -2593,15 +1964,15 @@
         <v>52</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="2" customFormat="1" ht="16">
+      <c r="A4" s="2" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>118</v>
+      <c r="B4" s="5" t="s">
+        <v>117</v>
       </c>
       <c r="C4" s="2">
         <v>1</v>
@@ -2610,18 +1981,18 @@
         <v>143</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" customFormat="1" ht="16">
+      <c r="A5" s="2" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" s="2" t="s">
-        <v>124</v>
-      </c>
       <c r="B5" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C5" s="2">
         <v>1</v>
@@ -2630,18 +2001,18 @@
         <v>143</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="F5" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" customFormat="1" ht="16">
+      <c r="A6" s="2" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="6" ht="14" customHeight="1" spans="1:6">
-      <c r="A6" s="2" t="s">
-        <v>127</v>
-      </c>
       <c r="B6" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C6" s="2">
         <v>1</v>
@@ -2650,58 +2021,58 @@
         <v>143</v>
       </c>
       <c r="E6" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" customFormat="1" ht="14" customHeight="1">
+      <c r="A7" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C7" s="2">
+        <v>1</v>
+      </c>
+      <c r="D7" s="2">
+        <v>143</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" s="2" t="s">
+    </row>
+    <row r="8" spans="1:6" customFormat="1" ht="16">
+      <c r="A8" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="C7" s="2">
-        <v>1</v>
-      </c>
-      <c r="D7" s="2">
+      <c r="C8" s="2">
+        <v>1</v>
+      </c>
+      <c r="D8" s="2">
         <v>406</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="8" ht="27" spans="1:6">
-      <c r="A8" s="2" t="s">
+    <row r="9" spans="1:6" customFormat="1" ht="32">
+      <c r="A9" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>132</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="C8" s="2">
-        <v>1</v>
-      </c>
-      <c r="D8" s="2">
-        <v>510</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>133</v>
       </c>
       <c r="C9" s="2">
         <v>1</v>
@@ -2710,18 +2081,18 @@
         <v>510</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>136</v>
+        <v>76</v>
       </c>
       <c r="F9" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" customFormat="1" ht="16">
+      <c r="A10" s="2" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" s="2" t="s">
-        <v>138</v>
-      </c>
       <c r="B10" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C10" s="2">
         <v>1</v>
@@ -2730,18 +2101,18 @@
         <v>510</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>52</v>
+        <v>135</v>
       </c>
       <c r="F10" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" customFormat="1" ht="16">
+      <c r="A11" s="2" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" s="2" t="s">
-        <v>140</v>
-      </c>
       <c r="B11" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C11" s="2">
         <v>1</v>
@@ -2750,18 +2121,18 @@
         <v>510</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="F11" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" customFormat="1" ht="16">
+      <c r="A12" s="2" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="12" spans="1:6">
-      <c r="A12" s="2" t="s">
-        <v>142</v>
-      </c>
       <c r="B12" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C12" s="2">
         <v>1</v>
@@ -2770,18 +2141,18 @@
         <v>510</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="F12" s="2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" customFormat="1" ht="16">
+      <c r="A13" s="2" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="13" spans="1:6">
-      <c r="A13" s="2" t="s">
-        <v>144</v>
-      </c>
       <c r="B13" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C13" s="2">
         <v>1</v>
@@ -2790,18 +2161,18 @@
         <v>510</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>125</v>
+        <v>22</v>
       </c>
       <c r="F13" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" customFormat="1" ht="16">
+      <c r="A14" s="2" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="14" ht="27" spans="1:6">
-      <c r="A14" s="2" t="s">
-        <v>146</v>
-      </c>
       <c r="B14" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C14" s="2">
         <v>1</v>
@@ -2810,18 +2181,18 @@
         <v>510</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>147</v>
+        <v>124</v>
       </c>
       <c r="F14" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" customFormat="1" ht="32">
+      <c r="A15" s="2" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="15" ht="81" spans="1:6">
-      <c r="A15" s="2" t="s">
-        <v>149</v>
-      </c>
       <c r="B15" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C15" s="2">
         <v>1</v>
@@ -2830,38 +2201,38 @@
         <v>510</v>
       </c>
       <c r="E15" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" customFormat="1" ht="96">
+      <c r="A16" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C16" s="2">
+        <v>1</v>
+      </c>
+      <c r="D16" s="2">
+        <v>510</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F15" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" s="2" t="s">
+      <c r="F16" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="16">
+      <c r="A17" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="C16" s="2">
-        <v>1</v>
-      </c>
-      <c r="D16" s="2">
-        <v>515</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="17" ht="27" spans="1:6">
-      <c r="A17" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>152</v>
       </c>
       <c r="C17" s="2">
         <v>1</v>
@@ -2870,18 +2241,18 @@
         <v>515</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="F17" s="2" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="32">
+      <c r="A18" s="2" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="18" spans="1:6">
-      <c r="A18" s="2" t="s">
-        <v>156</v>
-      </c>
       <c r="B18" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C18" s="2">
         <v>1</v>
@@ -2890,18 +2261,18 @@
         <v>515</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="F18" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="16">
+      <c r="A19" s="2" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="19" spans="1:6">
-      <c r="A19" s="2" t="s">
-        <v>158</v>
-      </c>
       <c r="B19" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C19" s="2">
         <v>1</v>
@@ -2910,18 +2281,18 @@
         <v>515</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>125</v>
+        <v>29</v>
       </c>
       <c r="F19" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="16">
+      <c r="A20" s="2" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="20" ht="27" spans="1:6">
-      <c r="A20" s="2" t="s">
-        <v>160</v>
-      </c>
       <c r="B20" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C20" s="2">
         <v>1</v>
@@ -2930,18 +2301,18 @@
         <v>515</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>147</v>
+        <v>124</v>
       </c>
       <c r="F20" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="32">
+      <c r="A21" s="2" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="21" spans="1:6">
-      <c r="A21" s="2" t="s">
-        <v>162</v>
-      </c>
       <c r="B21" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C21" s="2">
         <v>1</v>
@@ -2950,38 +2321,38 @@
         <v>515</v>
       </c>
       <c r="E21" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="16">
+      <c r="A22" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C22" s="2">
+        <v>1</v>
+      </c>
+      <c r="D22" s="2">
+        <v>515</v>
+      </c>
+      <c r="E22" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="F21" s="2" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="22" ht="27" spans="1:6">
-      <c r="A22" s="2" t="s">
+      <c r="F22" s="2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="32">
+      <c r="A23" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>164</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="C22" s="2">
-        <v>2</v>
-      </c>
-      <c r="D22" s="2">
-        <v>149</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="23" ht="27" spans="1:6">
-      <c r="A23" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>165</v>
       </c>
       <c r="C23" s="2">
         <v>2</v>
@@ -2990,18 +2361,18 @@
         <v>149</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>52</v>
+        <v>14</v>
       </c>
       <c r="F23" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="32">
+      <c r="A24" s="2" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="24" spans="1:6">
-      <c r="A24" s="2" t="s">
-        <v>169</v>
-      </c>
       <c r="B24" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C24" s="2">
         <v>2</v>
@@ -3010,18 +2381,18 @@
         <v>149</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="F24" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="16">
+      <c r="A25" s="2" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="25" ht="27" spans="1:6">
-      <c r="A25" s="2" t="s">
-        <v>171</v>
-      </c>
       <c r="B25" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C25" s="2">
         <v>2</v>
@@ -3030,18 +2401,18 @@
         <v>149</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>147</v>
+        <v>29</v>
       </c>
       <c r="F25" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="32">
+      <c r="A26" s="2" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="26" spans="1:6">
-      <c r="A26" s="2" t="s">
-        <v>173</v>
-      </c>
       <c r="B26" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C26" s="2">
         <v>2</v>
@@ -3050,38 +2421,38 @@
         <v>149</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>43</v>
+        <v>146</v>
       </c>
       <c r="F26" s="2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="16">
+      <c r="A27" s="2" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="27" spans="1:6">
-      <c r="A27" s="2" t="s">
-        <v>175</v>
-      </c>
       <c r="B27" s="2" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="C27" s="2">
         <v>2</v>
       </c>
       <c r="D27" s="2">
-        <v>185</v>
+        <v>149</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>125</v>
+        <v>43</v>
       </c>
       <c r="F27" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="16">
+      <c r="A28" s="2" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="28" ht="27" spans="1:6">
-      <c r="A28" s="2" t="s">
-        <v>178</v>
-      </c>
       <c r="B28" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C28" s="2">
         <v>2</v>
@@ -3090,18 +2461,18 @@
         <v>185</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>147</v>
+        <v>124</v>
       </c>
       <c r="F28" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="32">
+      <c r="A29" s="2" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="29" spans="1:6">
-      <c r="A29" s="2" t="s">
-        <v>180</v>
-      </c>
       <c r="B29" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C29" s="2">
         <v>2</v>
@@ -3110,18 +2481,18 @@
         <v>185</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>43</v>
+        <v>146</v>
       </c>
       <c r="F29" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="16">
+      <c r="A30" s="2" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="30" ht="27" spans="1:6">
-      <c r="A30" s="2" t="s">
-        <v>182</v>
-      </c>
       <c r="B30" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C30" s="2">
         <v>2</v>
@@ -3130,23 +2501,42 @@
         <v>185</v>
       </c>
       <c r="E30" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="32">
+      <c r="A31" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C31" s="2">
+        <v>2</v>
+      </c>
+      <c r="D31" s="2">
+        <v>185</v>
+      </c>
+      <c r="E31" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F30" s="2" t="s">
-        <v>183</v>
+      <c r="F31" s="2" t="s">
+        <v>182</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K1"/>
-  <sheetFormatPr defaultColWidth="8.83185840707965" defaultRowHeight="13.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="9" customWidth="1"/>
@@ -3162,7 +2552,7 @@
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -3189,23 +2579,21 @@
         <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>186</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultColWidth="8.83185840707965" defaultRowHeight="13.5" outlineLevelRow="7" outlineLevelCol="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="120" customWidth="1"/>
@@ -3213,70 +2601,69 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="B1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:2" ht="16">
+      <c r="A2" s="2" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="2" t="s">
+      <c r="B2" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="B2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:2" ht="16">
+      <c r="A3" s="2" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" s="2" t="s">
+      <c r="B3" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="B3" s="2" t="s">
+    </row>
+    <row r="4" spans="1:2" ht="16">
+      <c r="A4" s="2" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" s="2" t="s">
+      <c r="B4" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="B4" s="2" t="s">
+    </row>
+    <row r="5" spans="1:2" ht="16">
+      <c r="A5" s="2" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5" s="2" t="s">
+      <c r="B5" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="B5" s="2" t="s">
+    </row>
+    <row r="6" spans="1:2" ht="16">
+      <c r="A6" s="2" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" s="2" t="s">
+      <c r="B6" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="B6" s="2" t="s">
+    </row>
+    <row r="7" spans="1:2" ht="16">
+      <c r="A7" s="2" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="B7" s="2" t="s">
+    </row>
+    <row r="8" spans="1:2" ht="16">
+      <c r="A8" s="2" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="8" spans="1:2">
-      <c r="A8" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>201</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>202</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>